<commit_message>
Excel Chapter 3 learning and task completed
</commit_message>
<xml_diff>
--- a/3_Excel/Chapter_2_Arithemetic_and_Conditional_Operators/c2_task_1.xlsx
+++ b/3_Excel/Chapter_2_Arithemetic_and_Conditional_Operators/c2_task_1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROITBRIDGE_Learning\3_Excel\Chapter_2_Arithemetic_and_Conditional_Operators\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D0FF07B-D12C-43AC-8B7A-00D053E93604}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D090F51-9E30-42EC-97DF-7022E285B8B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -156,7 +156,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="[$₹-449]\ #,##0.00"/>
+    <numFmt numFmtId="164" formatCode="[$₹-449]\ #,##0.00"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -388,14 +388,14 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -404,7 +404,7 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -412,46 +412,46 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -981,170 +981,160 @@
       <c r="F13" s="4"/>
     </row>
     <row r="14" spans="1:15" ht="15.75" customHeight="1">
-      <c r="B14" s="24" t="s">
+      <c r="B14" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="25"/>
-      <c r="D14" s="25"/>
-      <c r="E14" s="26"/>
+      <c r="C14" s="35"/>
+      <c r="D14" s="35"/>
+      <c r="E14" s="36"/>
     </row>
     <row r="15" spans="1:15" ht="15.75" customHeight="1">
       <c r="B15" s="13" t="s">
         <v>26</v>
       </c>
       <c r="C15" s="14"/>
-      <c r="D15" s="17">
+      <c r="D15" s="26">
         <f>SUM(C2:C11)</f>
         <v>450</v>
       </c>
-      <c r="E15" s="18"/>
+      <c r="E15" s="28"/>
     </row>
     <row r="16" spans="1:15" ht="15.75" customHeight="1">
-      <c r="B16" s="17"/>
+      <c r="B16" s="26"/>
       <c r="C16" s="27"/>
       <c r="D16" s="27"/>
-      <c r="E16" s="18"/>
+      <c r="E16" s="28"/>
     </row>
     <row r="17" spans="2:5" ht="15.75" customHeight="1">
-      <c r="B17" s="24" t="s">
+      <c r="B17" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="C17" s="25"/>
-      <c r="D17" s="25"/>
-      <c r="E17" s="26"/>
+      <c r="C17" s="35"/>
+      <c r="D17" s="35"/>
+      <c r="E17" s="36"/>
     </row>
     <row r="18" spans="2:5" ht="15.75" customHeight="1">
-      <c r="B18" s="15" t="s">
+      <c r="B18" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="16"/>
-      <c r="D18" s="19">
+      <c r="C18" s="33"/>
+      <c r="D18" s="15">
         <f>MAX(E2:E11)</f>
         <v>624000</v>
       </c>
-      <c r="E18" s="20"/>
+      <c r="E18" s="16"/>
     </row>
     <row r="19" spans="2:5" ht="15.75" customHeight="1">
-      <c r="B19" s="17"/>
+      <c r="B19" s="26"/>
       <c r="C19" s="27"/>
       <c r="D19" s="27"/>
-      <c r="E19" s="18"/>
+      <c r="E19" s="28"/>
     </row>
     <row r="20" spans="2:5" ht="15.75" customHeight="1">
-      <c r="B20" s="24" t="s">
+      <c r="B20" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="26"/>
+      <c r="C20" s="35"/>
+      <c r="D20" s="35"/>
+      <c r="E20" s="36"/>
     </row>
     <row r="21" spans="2:5" ht="15.75" customHeight="1">
-      <c r="B21" s="15" t="s">
+      <c r="B21" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="C21" s="16"/>
-      <c r="D21" s="19">
+      <c r="C21" s="33"/>
+      <c r="D21" s="15">
         <f>MIN(E2:E11)</f>
         <v>16800</v>
       </c>
-      <c r="E21" s="20"/>
+      <c r="E21" s="16"/>
     </row>
     <row r="22" spans="2:5" ht="15.75" customHeight="1">
-      <c r="B22" s="28"/>
-      <c r="C22" s="29"/>
-      <c r="D22" s="29"/>
-      <c r="E22" s="30"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="30"/>
+      <c r="D22" s="30"/>
+      <c r="E22" s="31"/>
     </row>
     <row r="23" spans="2:5" ht="15.75" customHeight="1">
-      <c r="B23" s="21" t="s">
+      <c r="B23" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="23"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="25"/>
     </row>
     <row r="24" spans="2:5" ht="15.75" customHeight="1">
-      <c r="B24" s="15" t="s">
+      <c r="B24" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="C24" s="16"/>
-      <c r="D24" s="17">
-        <f>COUNTA(C2:C11)</f>
+      <c r="C24" s="33"/>
+      <c r="D24" s="26">
+        <f>COUNTA(B2:B11)</f>
         <v>10</v>
       </c>
-      <c r="E24" s="18"/>
+      <c r="E24" s="28"/>
     </row>
     <row r="25" spans="2:5" ht="15.75" customHeight="1">
-      <c r="B25" s="17"/>
+      <c r="B25" s="26"/>
       <c r="C25" s="27"/>
       <c r="D25" s="27"/>
-      <c r="E25" s="18"/>
+      <c r="E25" s="28"/>
     </row>
     <row r="26" spans="2:5" ht="15.75" customHeight="1">
-      <c r="B26" s="21" t="s">
+      <c r="B26" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="C26" s="22"/>
-      <c r="D26" s="22"/>
-      <c r="E26" s="23"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="25"/>
     </row>
     <row r="27" spans="2:5" ht="15.75" customHeight="1">
-      <c r="B27" s="15" t="s">
+      <c r="B27" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="C27" s="16"/>
-      <c r="D27" s="19">
+      <c r="C27" s="33"/>
+      <c r="D27" s="15">
         <f>AVERAGE(E2:E11)</f>
         <v>118865</v>
       </c>
-      <c r="E27" s="20"/>
+      <c r="E27" s="16"/>
     </row>
     <row r="28" spans="2:5" ht="15.75" customHeight="1">
-      <c r="B28" s="17"/>
+      <c r="B28" s="26"/>
       <c r="C28" s="27"/>
       <c r="D28" s="27"/>
-      <c r="E28" s="18"/>
+      <c r="E28" s="28"/>
     </row>
     <row r="29" spans="2:5" ht="15.75" customHeight="1">
-      <c r="B29" s="31" t="s">
+      <c r="B29" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="C29" s="32"/>
-      <c r="D29" s="32"/>
-      <c r="E29" s="33"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="18"/>
+      <c r="E29" s="19"/>
     </row>
     <row r="30" spans="2:5" ht="15.75" customHeight="1">
-      <c r="B30" s="34"/>
-      <c r="C30" s="35"/>
-      <c r="D30" s="35"/>
-      <c r="E30" s="36"/>
+      <c r="B30" s="20"/>
+      <c r="C30" s="21"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="22"/>
     </row>
     <row r="31" spans="2:5" ht="15.75" customHeight="1">
-      <c r="B31" s="17"/>
+      <c r="B31" s="26"/>
       <c r="C31" s="27"/>
       <c r="D31" s="27"/>
-      <c r="E31" s="18"/>
+      <c r="E31" s="28"/>
     </row>
     <row r="32" spans="2:5" ht="15.75" customHeight="1">
-      <c r="B32" s="21" t="s">
+      <c r="B32" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="C32" s="22"/>
-      <c r="D32" s="22"/>
-      <c r="E32" s="23"/>
+      <c r="C32" s="24"/>
+      <c r="D32" s="24"/>
+      <c r="E32" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="B29:E30"/>
-    <mergeCell ref="B32:E32"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="B19:E19"/>
-    <mergeCell ref="B22:E22"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="B28:E28"/>
-    <mergeCell ref="B31:E31"/>
-    <mergeCell ref="B27:C27"/>
     <mergeCell ref="B14:E14"/>
     <mergeCell ref="B17:E17"/>
     <mergeCell ref="B20:E20"/>
@@ -1157,6 +1147,16 @@
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="B24:C24"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="B29:E30"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="B27:C27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>